<commit_message>
Add Priority column: impact/effort quadrant for triaging low-hanging fruit
score_content.py: rubric prompt now also asks Claude to rate impact
(High/Low) and effort (High/Low) of the suggested fixes as a whole, for
any asset with suggestions. Priority is then computed deterministically
in Python from a fixed quadrant, not left to the model to self-label, so
it's applied consistently across every asset:
  High impact + Low effort  -> Quick Win       (do these first)
  High impact + High effort -> Major Project
  Low impact + Low effort   -> Fill-In
  Low impact + High effort  -> Low Priority

Dashboard: new Priority column (sortable, filterable), a 'Quick wins'
stat tile, and Impact/Effort shown in each item's expanded detail.

Verified against the real 4-item sample via the live API.
</commit_message>
<xml_diff>
--- a/data/scored_sample-preview.xlsx
+++ b/data/scored_sample-preview.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,6 +484,21 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>Last Audited</t>
         </is>
       </c>
@@ -509,7 +524,7 @@
         <v>9</v>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" t="n">
         <v>10</v>
@@ -521,7 +536,7 @@
         <v>12</v>
       </c>
       <c r="J2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -530,19 +545,34 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>The biggest weakness is SEO — there is no meta description, no structured H2/H3 hierarchy beyond a single 'The Solution' header, and keyword targeting for high-value terms like 'after-hours HVAC software' or 'on-demand HVAC for commercial buildings' is absent. The biggest strength is a logical problem-solution narrative with a real CTA (demo link) at the end.</t>
+          <t>The biggest weakness is SEO: there is no meta description, the title is functional but unoptimized, headers are plain sentences rather than keyword-rich H2/H3s, and there are no internal links to related Genea content or product pages. The biggest strength is a clear problem-solution narrative with a logical flow and an explicit demo CTA at the end.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>- Add a meta description targeting 'after-hours HVAC software for commercial buildings' — none currently exists, which is the single highest-impact SEO gap for a crawlable blog post.
-- Restructure the four problem paragraphs as explicit H2s (e.g., 'Problem 1: Tenants Rarely Have 24–48 Hours of Advance Notice,' 'Problem 2: No Cancellation Flexibility Wastes Energy and Money') to create a scannable header hierarchy and capture featured-snippet opportunities for queries like 'problems with work order systems for HVAC.'
-- Fix copy errors that undermine credibility: 'the all parties,' 'submit a request in with the click,' 'are able so specify,' and the broken anchor text 'the amount of billing leakage can be substantia l' should all be corrected before the page is re-indexed.
-- Replace the vague first-person closing ('reach out to me') with a brand-consistent CTA tied to Genea's On-Demand HVAC product page — the anonymous 'me' reference makes the content feel like a personal LinkedIn post rather than a company asset and breaks trust for cold traffic.
-- Add at least two internal links — one to Genea's core access control or smart building platform page and one to a relevant case study or ROI/billing-leakage data page — to distribute link equity and give readers a next step beyond the demo form.</t>
+          <t>- Add a meta description targeting 'on-demand HVAC software for commercial buildings' or 'after-hours HVAC request management' — none currently exists, which leaves a high-value SERP snippet slot blank.
+- Rewrite the four section headers (e.g., 'On-Demand HVAC requests require advanced notice that tenants don't have') into keyword-rich H2s such as 'Why After-Hours HVAC Requests Fail Without Advance Notice' to improve crawlability and target long-tail queries around 'after hours HVAC requests.'
+- Replace first-person 'reach out to me' CTA with a brand-consistent CTA such as 'Request a demo of Genea On-Demand HVAC' — the current phrasing reads as a personal sales email rather than a scalable SaaS product page and undermines brand credibility.
+- Fix the typo 'are able so specify' (should be 'to specify') and the broken anchor text 'the amount of billing leakage can be substantia l' (split word), as these grammar errors reduce trust and readability for a SaaS buyer audience.
+- Add 2-3 internal links to related Genea content (e.g., a product page for On-Demand HVAC, a case study on billing leakage, or a blog post on BMS integrations) to distribute page authority and guide prospects deeper into the funnel — currently zero internal links exist beyond the two 'On-Demand HVAC service' anchors, which both appear to point to the same destination.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Quick Win</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
@@ -566,22 +596,22 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" t="n">
         <v>11</v>
       </c>
-      <c r="G3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>10</v>
       </c>
-      <c r="I3" t="n">
-        <v>9</v>
-      </c>
       <c r="J3" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -590,19 +620,34 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>The biggest issue is severe staleness — no last-updated date, OfferUp's market position description reads as circa 2018-2019 and may no longer be accurate, and the phrase 'cloud-based access control' conflicts with Genea's current 'cloud-native' positioning; the biggest strength is a clear, specific CTA tied to a named integration (Okta Lifecycle Management) that gives conversion context.</t>
+          <t>The biggest issue is severe staleness — OfferUp's company status, Genea's product naming ('cloud-based access control' rather than current positioning language), and a missing Last Updated date all signal this content may be years old and could actively mislead prospects. The biggest strength is a clear, relevant use-case hook around Okta Lifecycle Management integration, which is a high-value keyword and a genuine differentiator for Genea.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>- Replace 'cloud-based access control solution' with 'cloud-native access control' throughout to match Genea's current brand positioning and avoid contradicting the company's core differentiator messaging.
-- Verify and update all OfferUp company facts — 'largest mobile marketplace,' 'top five most popular shopping apps for over three years,' and the Bellevue HQ claim are likely stale and could damage credibility if inaccurate; rewrite the intro paragraph with confirmed current figures or remove specific superlatives.
-- Add a meta description targeting a keyword phrase such as 'Okta access control integration case study' — none currently exists, and this page has strong long-tail SEO potential given the named Okta Lifecycle Management integration.
-- Expand the body content beyond the current three-sentence summary: add at least one quantified outcome (e.g., provisioning time reduced by X%, number of employees managed) to give the case study credibility and improve time-on-page metrics.
-- Add an H1 distinct from the page title and introduce subheaders (e.g., 'The Challenge,' 'The Solution,' 'The Results') to improve header structure for both SEO crawlability and reader navigation.</t>
+          <t>- Verify and update OfferUp's current company status and description — OfferUp went through significant changes (merger with Letgo in 2020) and describing it as 'rapidly growing' with 'top five' app rankings that are undated will undermine credibility with prospects doing due diligence.
+- Replace 'cloud-based access control solution' throughout with Genea's current brand language (e.g., 'cloud-native access control') and add the current product name (Genea Access Control) to align with present positioning and avoid appearing out of date.
+- Add a meta description targeting a phrase such as 'Okta access control integration case study' — none currently exists, and the Okta Lifecycle Management angle is a high-intent, differentiating keyword that is completely absent from any SEO metadata.
+- Expand the body content beyond four sentences — case studies at this length cannot rank, build trust, or move a prospect through the funnel; add a Challenge / Solution / Results structure with at least one quantified outcome (e.g., provisioning time reduction) sourced from OfferUp.
+- Fix the typo 'Belleuve' (should be 'Bellevue') in the opening line, and add a Last Updated date to the page to signal freshness to both readers and search engines.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
@@ -626,22 +671,22 @@
         </is>
       </c>
       <c r="E4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H4" t="n">
         <v>5</v>
       </c>
-      <c r="F4" t="n">
-        <v>10</v>
-      </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>8</v>
       </c>
-      <c r="H4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I4" t="n">
-        <v>7</v>
-      </c>
       <c r="J4" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -650,19 +695,34 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>The page is almost entirely navigation chrome and boilerplate with virtually no substantive body content describing the braXos integration — there is no meta description, no meaningful H2/H3 structure, no keyword-rich copy, and no explanation of what the integration actually does or why a buyer should care. The one strength is that a 'Book A Demo' CTA is present and the integration category (Access Control + Visitor Management + Elevator Controls) is at least labeled.</t>
+          <t>The page is essentially a shell — it contains almost no substantive body copy about what the Genea + braXos integration actually does, how it works, or why a buyer should care, making it nearly worthless for SEO and conversion. The one strength is that a 'Book A Demo' CTA and basic navigation structure are present.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>- Write a minimum 300-word body section explaining exactly what the Genea + braXos destination dispatch integration does — which hardware is supported, how elevator access ties to credential events, and what problem it solves for commercial real estate or enterprise customers — because right now there is zero descriptive content on the page.
-- Add a meta description targeting a phrase such as 'cloud-based access control elevator destination dispatch integration' since none currently exists, which will prevent search engines from auto-generating an uncontrolled snippet and will suppress click-through rates.
-- Replace the vague H1 'Integrated Access Control and Visitor Management and Elevator Controls' with a benefit-led headline such as 'Automate Elevator Access with Genea + braXos Destination Dispatch — No Proprietary Hardware Required' to align with Genea's cloud-native, hardware-agnostic positioning and improve keyword relevance.
-- Add 2-3 structured H2 sections (e.g., 'How the Integration Works,' 'Key Features,' 'Supported Use Cases') with real copy beneath each, since the current page has no header hierarchy below the H1, making it unfavorable for both crawlers and readers.
-- Include at least one internal link to the Genea Security product page and one to the Integrations directory page to distribute page authority and give visitors a clear path deeper into the site — neither link currently exists in the body content.</t>
+          <t>- Write a minimum 300-word body describing exactly what the Genea + braXos destination dispatch integration does (e.g., how access credentials trigger elevator calls, which hardware is supported, which Genea product tiers include it) — the current page has zero explanatory content, which tanks SEO and conversion.
+- Add a meta description and rewrite the H1 from 'Genea + braXos' to something keyword-rich like 'Genea Access Control + braXos Destination Dispatch Elevator Integration' to give search engines a clear signal for queries around 'access control elevator integration' or 'destination dispatch access control.'
+- Add a structured 'How It Works' section with 3–4 steps or a diagram showing the data flow between Genea's cloud platform and the braXos elevator controller, directly addressing the buyer question this page must answer before they book a demo.
+- Replace the generic tagline 'Your ticket to the cloud is here' (which reads as a nav/footer bleed-in, not page body copy) with a value-proposition sentence specific to the integration, such as how unified access and elevator control reduces friction for tenants and simplifies administration for property managers.
+- Add 2–3 internal links to relevant Genea pages (e.g., the Visitor Management product page, Commercial Real Estate industry page, or the main Integrations hub) to pass link equity and guide users deeper into the funnel — currently no in-content links exist.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
@@ -710,19 +770,34 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>The page's biggest weakness is pervasive staleness — the Apache Log4j2 CVE-2021-44228 section reads as a live incident response from late 2021, severely undermining trust on a security-focused page; the biggest strength is that it covers a broad range of genuine compliance topics (SOC 2, GDPR, CCPA, UL, encryption standards) that prospects actively search for.</t>
+          <t>The page's biggest weakness is a cluster of staleness and accuracy issues — most visibly the Apache Log4j2 section, which references a 2021 CVE as an active investigation, making the page read as years out of date and potentially eroding trust on a page specifically dedicated to security credibility. The biggest strength is reasonable coverage of compliance topics (SOC 2, GDPR, CCPA, technical controls) that gives prospects a solid checklist-style reference.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>- Remove or archive the Apache Log4j2 CVE-2021-44228 incident-response section entirely — leaving a 2021 emergency notice on a security compliance page in 2025/2026 signals the page is unmaintained and erodes trust with security-conscious buyers.
-- Add a proper meta description targeting high-intent queries such as 'cloud access control SOC 2 GDPR compliance' — none currently exists, and the page title 'Genea | Security and Compliance Regulations' is too generic to differentiate or rank competitively.
-- Replace the vague inline CTA ('Your ticket to the cloud is here. Talk to a Genea Expert, today') with a dedicated, compliance-specific CTA such as 'Request our SOC 2 Type 2 report or schedule a security review with a Genea expert' to match the decision-stage intent of visitors on this page.
-- Fix the typo 'OWSP top10' (should be 'OWASP Top 10') and rewrite the awkward sentence in the Data in Transit section ('Anyone or anything, including a supercomputer that attempts to pry, may take years to crack...') — on a security compliance page, unprofessional copy damages credibility with IT and security buyers.
-- Add H2/H3 structured headers that include keyword-rich phrases (e.g., 'SOC 2 Type 2 Certification', 'GDPR Compliance for Access Control') and cross-link to relevant product pages (Security, IT and Security Teams role page) to improve crawlability and internal link equity.</t>
+          <t>- Remove or archive the Apache Log4j2 section entirely — leaving a 2021 CVE investigation notice live on a security-and-compliance page signals the site is unmaintained and directly undercuts trust; if retained, reframe it as a resolved historical incident with a closing date.
+- Add a meta description targeting terms like 'cloud access control security compliance SOC 2 GDPR' — no meta description currently exists, which wastes a high-intent page that prospects and enterprise security reviewers actively search for.
+- Replace the generic CTA 'Your ticket to the cloud is here. Talk to a Genea Expert, today' with a compliance-specific CTA such as 'Request our SOC 2 Type 2 report or book a security review with a Genea expert' — the current CTA ignores the security-buyer context and misses the explicit report-request action already mentioned in the SOC 2 body copy.
+- Fix the typo 'OWSP top10' (should be 'OWASP Top 10') in the Vulnerability Assessment section and rewrite the sentence 'Genea also employs an in-house network security team who run manual and automated vulnerability assessment and penetration tests time to time' — both errors on a security-credibility page damage brand trust with technical buyers.
+- Add an H2 or callout confirming the last-reviewed or last-updated date for compliance certifications (e.g., 'SOC 2 Type 2 last audited: [Year]') so enterprise and Fortune 50 prospects — called out in the intro copy — can confirm the information is current without contacting sales.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Quick Win</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>

</xml_diff>